<commit_message>
Rewrite AL section B in plain language with examples
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DzTYgXHQRdW29cqRnE8XYg
</commit_message>
<xml_diff>
--- a/Control_Stage_AL.xlsx
+++ b/Control_Stage_AL.xlsx
@@ -2977,7 +2977,7 @@
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="66" t="inlineStr">
         <is>
-          <t>B. LR SLOT — three lanes, hazards, register state</t>
+          <t>B. LR SLOT — the 3 lanes working together: what each lane sees, when a new value becomes visible, and reset</t>
         </is>
       </c>
       <c r="B32" s="67" t="n"/>
@@ -3001,17 +3001,17 @@
       </c>
       <c r="C33" s="70" t="inlineStr">
         <is>
-          <t>The module shall execute any LR opcode in any lane, with up to three LR sub-instructions in parallel in one word.</t>
+          <t>Each VLIW word has 3 LR lanes. The module shall execute any LR op in any lane, all lanes in the same cycle.</t>
         </is>
       </c>
       <c r="D33" s="70" t="inlineStr">
         <is>
-          <t>Lanes are identical. ADDB/ADDBI write two LRs each (Spec Questions Q4); unused lane encoding — Q7.</t>
+          <t>Plain words: one instruction word can carry up to 3 LR commands (e.g. lane0 = INC LR1, lane1 = SET LR2, lane2 = SUB LR3). Any command may sit in any lane. A lane may also be empty (NOP) — how an empty lane is encoded is Spec Question Q7.</t>
         </is>
       </c>
       <c r="E33" s="70" t="inlineStr">
         <is>
-          <t>Random opcode / lane mix, 1..3 active lanes, distinct dests  [standard]</t>
+          <t>Random words: random command in each lane, 1 to 3 lanes used, all destinations different  [standard]</t>
         </is>
       </c>
       <c r="F33" s="71" t="inlineStr">
@@ -3042,7 +3042,7 @@
       <c r="D34" s="76" t="n"/>
       <c r="E34" s="70" t="inlineStr">
         <is>
-          <t>All lanes NOP, and partially NOP words  [corner]</t>
+          <t>Words with empty lanes (all 3 empty, or only some)  [corner]</t>
         </is>
       </c>
       <c r="F34" s="71" t="inlineStr">
@@ -3066,14 +3066,14 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
+    <row r="35" ht="33" customHeight="1">
       <c r="A35" s="77" t="n"/>
       <c r="B35" s="77" t="n"/>
       <c r="C35" s="77" t="n"/>
       <c r="D35" s="77" t="n"/>
       <c r="E35" s="70" t="inlineStr">
         <is>
-          <t>Several ADDB / ADDBI pairs in one word  [corner]</t>
+          <t>Words with several ADDB/ADDBI in one word (each one writes 2 registers, so up to 6 registers change — Q4)  [corner]</t>
         </is>
       </c>
       <c r="F35" s="71" t="inlineStr">
@@ -3097,7 +3097,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="46" customHeight="1">
+    <row r="36" ht="85" customHeight="1">
       <c r="A36" s="72" t="inlineStr">
         <is>
           <t>LAN-02</t>
@@ -3110,17 +3110,17 @@
       </c>
       <c r="C36" s="74" t="inlineStr">
         <is>
-          <t>The module shall read all lane source operands from the prior-cycle snapshot, not from another lane's result in the same word.</t>
+          <t>All lanes shall read their input registers as they were at the START of the cycle, never the result of another lane in the same word.</t>
         </is>
       </c>
       <c r="D36" s="74" t="inlineStr">
         <is>
-          <t>Spec §5.</t>
+          <t>Example word: lane0 = INC LR1 5, lane1 = ADD LR2 LR1 CR0. Lane1 must use the OLD LR1 (before +5), because lane0's write only becomes visible in the next word. Another example: lane0 = ADD LR0 LR1 CR0 and lane1 = ADD LR1 LR0 CR0 in one word swaps the two registers.</t>
         </is>
       </c>
       <c r="E36" s="74" t="inlineStr">
         <is>
-          <t>Words where one lane reads an LR another lane writes (any lane pair, any opcode), incl. register swap / rotate in one word  [corner]</t>
+          <t>Random words where one lane reads a register that another lane writes in the same word (any lane pair, any command)  [corner]</t>
         </is>
       </c>
       <c r="F36" s="75" t="inlineStr">
@@ -3144,7 +3144,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="33" customHeight="1">
+    <row r="37" ht="46" customHeight="1">
       <c r="A37" s="68" t="inlineStr">
         <is>
           <t>LAN-03</t>
@@ -3157,17 +3157,17 @@
       </c>
       <c r="C37" s="70" t="inlineStr">
         <is>
-          <t>The module shall change only the destination registers named in the word.</t>
+          <t>The module shall change only the registers that the word writes. All other LRs keep their value.</t>
         </is>
       </c>
       <c r="D37" s="70" t="inlineStr">
         <is>
-          <t>Full 16-LR compare every cycle.</t>
+          <t>Checker rule, not a special stimulus: after every cycle compare all 16 LRs with the reference model.</t>
         </is>
       </c>
       <c r="E37" s="70" t="inlineStr">
         <is>
-          <t>All 16 LRs checked each cycle over random programs  [standard]</t>
+          <t>Compare all 16 LRs every cycle during the random runs of the other rows  [standard]</t>
         </is>
       </c>
       <c r="F37" s="71" t="inlineStr">
@@ -3191,7 +3191,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="46" customHeight="1">
+    <row r="38" ht="59" customHeight="1">
       <c r="A38" s="72" t="inlineStr">
         <is>
           <t>TIM-01</t>
@@ -3204,13 +3204,17 @@
       </c>
       <c r="C38" s="74" t="inlineStr">
         <is>
-          <t>The module shall make an LR written in word N visible to LR-ALU sources in words N+1 and later.</t>
-        </is>
-      </c>
-      <c r="D38" s="74" t="n"/>
+          <t>A value written to an LR in word N shall be usable by the LR lanes in word N+1 (and any later word), with no gap.</t>
+        </is>
+      </c>
+      <c r="D38" s="74" t="inlineStr">
+        <is>
+          <t>Example: word N: SET LR3 #5. Word N+1: ADD LR4 LR3 CR1 must see LR3 = 5. This is the most common pattern in real code (counters, pointers), so it must work back-to-back.</t>
+        </is>
+      </c>
       <c r="E38" s="74" t="inlineStr">
         <is>
-          <t>Random dependent chains: producer op, consumer op, lane and distance 1..N randomized  [standard]</t>
+          <t>Random chains of words where each word uses a register written 1, 2, 3 … words earlier; random command in producer and consumer  [standard]</t>
         </is>
       </c>
       <c r="F38" s="75" t="inlineStr">
@@ -3234,7 +3238,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="46" customHeight="1">
+    <row r="39" ht="72" customHeight="1">
       <c r="A39" s="68" t="inlineStr">
         <is>
           <t>TIM-02</t>
@@ -3247,17 +3251,17 @@
       </c>
       <c r="C39" s="70" t="inlineStr">
         <is>
-          <t>The module shall evaluate branch operands (reg1, reg2, BR reg) from the prior-cycle snapshot.</t>
+          <t>A branch shall compare the register values as they were at the START of the cycle (the same rule as LAN-02).</t>
         </is>
       </c>
       <c r="D39" s="70" t="inlineStr">
         <is>
-          <t>Spec §5 / §10.</t>
+          <t>Example: word N: DEC LR0 1 together with BNE LR0 CR0 loop. The branch looks at LR0 BEFORE the DEC, not after. A DEC in the word BEFORE the branch is seen. Getting this wrong makes every loop run one iteration too many or too few.</t>
         </is>
       </c>
       <c r="E39" s="70" t="inlineStr">
         <is>
-          <t>LR written in the same word as the branch (old value used) or the word before (new value used), biased so the write flips the outcome  [corner]</t>
+          <t>Random branch words with an LR write to the compared register in the same word (old value must be used) or in the word before (new value must be used); stimulus biased so that old vs new gives a different taken / not-taken result  [corner]</t>
         </is>
       </c>
       <c r="F39" s="71" t="inlineStr">
@@ -3281,7 +3285,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="59" customHeight="1">
+    <row r="40" ht="98" customHeight="1">
       <c r="A40" s="72" t="inlineStr">
         <is>
           <t>TIM-03</t>
@@ -3294,17 +3298,17 @@
       </c>
       <c r="C40" s="74" t="inlineStr">
         <is>
-          <t>The module shall execute the slots of the branch word itself in both outcomes, and shall give the non-selected fetch candidate no side effect (LR write, load, bus).</t>
+          <t>At a branch the chip fetches both the next word and the branch target. Only the chosen word may have any effect; the other one shall have none.</t>
         </is>
       </c>
       <c r="D40" s="74" t="inlineStr">
         <is>
-          <t>PC+1 and label are fetched in parallel; only one may execute.</t>
+          <t>Example: BEQ … target. The word at PC+1 holds INC LR5, the word at the target holds INC LR6. If the branch is taken, LR5 must NOT change; if not taken, LR6 must NOT change. The same for loads and the other stage slots. The branch word's own LR / load / stage slots always run, taken or not.</t>
         </is>
       </c>
       <c r="E40" s="74" t="inlineStr">
         <is>
-          <t>Taken and not-taken branches whose both candidate words carry LR writes / loads / bus slots  [corner]</t>
+          <t>Random branches (taken and not taken) where both candidate words carry LR writes, loads and stage slots  [corner]</t>
         </is>
       </c>
       <c r="F40" s="75" t="inlineStr">
@@ -3328,7 +3332,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="46" customHeight="1">
+    <row r="41" ht="59" customHeight="1">
       <c r="A41" s="68" t="inlineStr">
         <is>
           <t>LRF-01</t>
@@ -3341,17 +3345,17 @@
       </c>
       <c r="C41" s="70" t="inlineStr">
         <is>
-          <t>The module shall keep 16 independent 32-bit LRs, treat LRDn as an alias of LR(n+1):LR(n), and read CR0 / CR1 as 0 / 1.</t>
+          <t>The module shall keep the 16 LRs as separate 32-bit registers; LRDn is only another name for the pair LR(n+1):LR(n); CR0 always reads 0 and CR1 always reads 1.</t>
         </is>
       </c>
       <c r="D41" s="70" t="inlineStr">
         <is>
-          <t>LR0 is an ordinary register.</t>
+          <t>Example: write LR2 and LR3 separately, then ADDB LRD2 must work on their combined 64 bits; after ADDB LRD2, reading LR2 / LR3 shows the new bytes.</t>
         </is>
       </c>
       <c r="E41" s="70" t="inlineStr">
         <is>
-          <t>Random mix of scalar and pair accesses across all LRs and CRs  [standard]</t>
+          <t>Random programs mixing single-register and pair (LRD) access across all LRs and CRs  [standard]</t>
         </is>
       </c>
       <c r="F41" s="71" t="inlineStr">
@@ -3375,7 +3379,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="33" customHeight="1">
+    <row r="42" ht="46" customHeight="1">
       <c r="A42" s="72" t="inlineStr">
         <is>
           <t>LRF-02</t>
@@ -3388,17 +3392,17 @@
       </c>
       <c r="C42" s="74" t="inlineStr">
         <is>
-          <t>The module shall restart at PC 0 and drop pending LR writes when rst is asserted.</t>
+          <t>On reset the module shall go back to PC 0 and throw away any LR writes that were still in progress.</t>
         </is>
       </c>
       <c r="D42" s="74" t="inlineStr">
         <is>
-          <t>LR reset value is not specified — Spec Questions Q6.</t>
+          <t>Reset value of the LRs is not written in the spec (Q6), so only the PC / no-late-write part can be checked now.</t>
         </is>
       </c>
       <c r="E42" s="74" t="inlineStr">
         <is>
-          <t>Reset at a random time: mid-kernel, in a branch cycle, after HALT; short and long pulse  [corner]</t>
+          <t>Reset applied at a random moment: in the middle of a program, in the cycle of a branch, after HALT; short and long pulses  [corner]</t>
         </is>
       </c>
       <c r="F42" s="75" t="inlineStr">

</xml_diff>

<commit_message>
Fix V/X conditional formatting colors (green/red)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DzTYgXHQRdW29cqRnE8XYg
</commit_message>
<xml_diff>
--- a/Control_Stage_AL.xlsx
+++ b/Control_Stage_AL.xlsx
@@ -700,16 +700,26 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -717,6 +727,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00F8CBAD"/>
+          <bgColor rgb="00F8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -724,6 +735,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFE699"/>
+          <bgColor rgb="00FFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -731,6 +743,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00C6E0B4"/>
+          <bgColor rgb="00C6E0B4"/>
         </patternFill>
       </fill>
     </dxf>

</xml_diff>

<commit_message>
Add static green/red/priority fills so colors show in viewers without conditional formatting
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DzTYgXHQRdW29cqRnE8XYg
</commit_message>
<xml_diff>
--- a/Control_Stage_AL.xlsx
+++ b/Control_Stage_AL.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -120,6 +120,30 @@
     <font>
       <name val="Arial"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00833C0B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
       <sz val="10"/>
     </font>
     <font>
@@ -408,7 +432,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -532,7 +556,7 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -558,7 +582,7 @@
     <xf numFmtId="0" fontId="9" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -604,7 +628,10 @@
     <xf numFmtId="0" fontId="11" fillId="22" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="22" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -616,14 +643,17 @@
     <xf numFmtId="0" fontId="11" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2100,12 +2130,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G7" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H7" s="71" t="inlineStr">
+      <c r="G7" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H7" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2117,42 +2147,42 @@
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
-      <c r="A8" s="72" t="inlineStr">
+      <c r="A8" s="73" t="inlineStr">
         <is>
           <t>SYS-02</t>
         </is>
       </c>
-      <c r="B8" s="73" t="inlineStr">
+      <c r="B8" s="74" t="inlineStr">
         <is>
           <t>System assumptions</t>
         </is>
       </c>
-      <c r="C8" s="74" t="inlineStr">
+      <c r="C8" s="75" t="inlineStr">
         <is>
           <t>Programs are legal: no two lanes write the same LR (ADDB/ADDBI write both LR(n) and LR(n+1)); INC.MODP2 k in 1..9; LRD index even; branch / BR targets inside the active bank.</t>
         </is>
       </c>
-      <c r="D8" s="74" t="inlineStr">
+      <c r="D8" s="75" t="inlineStr">
         <is>
           <t>Spec §10.1. What the hardware does on illegal programs is not specified — Spec Questions Q5, Q9, Q12.</t>
         </is>
       </c>
-      <c r="E8" s="74" t="inlineStr">
+      <c r="E8" s="75" t="inlineStr">
         <is>
           <t>Assumption — environment constraints, not stimulated</t>
         </is>
       </c>
-      <c r="F8" s="75" t="inlineStr">
+      <c r="F8" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G8" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H8" s="75" t="inlineStr">
+      <c r="G8" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H8" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2194,12 +2224,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G9" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H9" s="71" t="inlineStr">
+      <c r="G9" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H9" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2211,42 +2241,42 @@
       </c>
     </row>
     <row r="10" ht="33" customHeight="1">
-      <c r="A10" s="72" t="inlineStr">
+      <c r="A10" s="73" t="inlineStr">
         <is>
           <t>SYS-04</t>
         </is>
       </c>
-      <c r="B10" s="73" t="inlineStr">
+      <c r="B10" s="74" t="inlineStr">
         <is>
           <t>System assumptions</t>
         </is>
       </c>
-      <c r="C10" s="74" t="inlineStr">
+      <c r="C10" s="75" t="inlineStr">
         <is>
           <t>Downstream stages and XMEM never back-pressure CTRL.</t>
         </is>
       </c>
-      <c r="D10" s="74" t="inlineStr">
+      <c r="D10" s="75" t="inlineStr">
         <is>
           <t>Memory-wait behavior is not updated in the spec — see group MEM.</t>
         </is>
       </c>
-      <c r="E10" s="74" t="inlineStr">
+      <c r="E10" s="75" t="inlineStr">
         <is>
           <t>Assumption — remove when the memory-wait spec is released</t>
         </is>
       </c>
-      <c r="F10" s="75" t="inlineStr">
+      <c r="F10" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G10" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H10" s="75" t="inlineStr">
+      <c r="G10" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H10" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2302,12 +2332,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G12" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H12" s="71" t="inlineStr">
+      <c r="G12" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H12" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2333,12 +2363,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G13" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H13" s="71" t="inlineStr">
+      <c r="G13" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H13" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2359,17 +2389,17 @@
           <t>Boundary class: CR0 / CR1 / CR15, imm min / max / -1, mode-bit boundary  [corner]</t>
         </is>
       </c>
-      <c r="F14" s="71" t="inlineStr">
+      <c r="F14" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G14" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H14" s="71" t="inlineStr">
+      <c r="G14" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H14" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2381,42 +2411,42 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="72" t="inlineStr">
+      <c r="A15" s="73" t="inlineStr">
         <is>
           <t>ADS-01</t>
         </is>
       </c>
-      <c r="B15" s="73" t="inlineStr">
+      <c r="B15" s="74" t="inlineStr">
         <is>
           <t>LR ops: ADD / SUB</t>
         </is>
       </c>
-      <c r="C15" s="74" t="inlineStr">
+      <c r="C15" s="75" t="inlineStr">
         <is>
           <t>The module shall write (src_a + src_b)[31:0] into dest when ADD is issued (src_b = LR or CR).</t>
         </is>
       </c>
-      <c r="D15" s="74" t="inlineStr">
+      <c r="D15" s="75" t="inlineStr">
         <is>
           <t>32-bit wrap, no saturation, no flags.</t>
         </is>
       </c>
-      <c r="E15" s="74" t="inlineStr">
+      <c r="E15" s="75" t="inlineStr">
         <is>
           <t>Random sources (LR / CR mix) and dest  [standard]</t>
         </is>
       </c>
-      <c r="F15" s="75" t="inlineStr">
+      <c r="F15" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G15" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H15" s="75" t="inlineStr">
+      <c r="G15" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H15" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2432,22 +2462,22 @@
       <c r="B16" s="76" t="n"/>
       <c r="C16" s="76" t="n"/>
       <c r="D16" s="76" t="n"/>
-      <c r="E16" s="74" t="inlineStr">
+      <c r="E16" s="75" t="inlineStr">
         <is>
           <t>Operands biased to wrap points (0, ±1, 0x7FFFFFFF, 0x80000000, 0xFFFFFFFF)  [corner]</t>
         </is>
       </c>
-      <c r="F16" s="75" t="inlineStr">
+      <c r="F16" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G16" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H16" s="75" t="inlineStr">
+      <c r="G16" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H16" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2463,22 +2493,22 @@
       <c r="B17" s="77" t="n"/>
       <c r="C17" s="77" t="n"/>
       <c r="D17" s="77" t="n"/>
-      <c r="E17" s="74" t="inlineStr">
+      <c r="E17" s="75" t="inlineStr">
         <is>
           <t>Operand aliasing: dest == src_a / src_b, src_a == src_b  [corner]</t>
         </is>
       </c>
-      <c r="F17" s="75" t="inlineStr">
+      <c r="F17" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G17" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H17" s="75" t="inlineStr">
+      <c r="G17" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H17" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2520,12 +2550,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G18" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H18" s="71" t="inlineStr">
+      <c r="G18" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H18" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2551,12 +2581,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G19" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H19" s="71" t="inlineStr">
+      <c r="G19" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H19" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2577,17 +2607,17 @@
           <t>Operand aliasing (loop-counter form SUB LRx LRx CR1)  [corner]</t>
         </is>
       </c>
-      <c r="F20" s="71" t="inlineStr">
+      <c r="F20" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G20" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H20" s="71" t="inlineStr">
+      <c r="G20" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H20" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2599,42 +2629,42 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="72" t="inlineStr">
+      <c r="A21" s="73" t="inlineStr">
         <is>
           <t>MOD-01</t>
         </is>
       </c>
-      <c r="B21" s="73" t="inlineStr">
+      <c r="B21" s="74" t="inlineStr">
         <is>
           <t>LR op: INC.MODP2</t>
         </is>
       </c>
-      <c r="C21" s="74" t="inlineStr">
+      <c r="C21" s="75" t="inlineStr">
         <is>
           <t>The module shall write (dst + step) &amp; ((1&lt;&lt;k)-1) into dst when INC.MODP2 is issued.</t>
         </is>
       </c>
-      <c r="D21" s="74" t="inlineStr">
+      <c r="D21" s="75" t="inlineStr">
         <is>
           <t>k 1..9 (encoded k-1). step is a signed 32-bit LR or CR value.</t>
         </is>
       </c>
-      <c r="E21" s="74" t="inlineStr">
+      <c r="E21" s="75" t="inlineStr">
         <is>
           <t>Random k, dst, step (all inside the mask)  [standard]</t>
         </is>
       </c>
-      <c r="F21" s="75" t="inlineStr">
+      <c r="F21" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G21" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H21" s="75" t="inlineStr">
+      <c r="G21" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H21" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2650,22 +2680,22 @@
       <c r="B22" s="76" t="n"/>
       <c r="C22" s="76" t="n"/>
       <c r="D22" s="76" t="n"/>
-      <c r="E22" s="74" t="inlineStr">
+      <c r="E22" s="75" t="inlineStr">
         <is>
           <t>Wrap class: sum at / around 2^k, negative and large steps, dst already above the mask  [corner]</t>
         </is>
       </c>
-      <c r="F22" s="75" t="inlineStr">
+      <c r="F22" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G22" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H22" s="75" t="inlineStr">
+      <c r="G22" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H22" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2681,22 +2711,22 @@
       <c r="B23" s="76" t="n"/>
       <c r="C23" s="76" t="n"/>
       <c r="D23" s="76" t="n"/>
-      <c r="E23" s="74" t="inlineStr">
+      <c r="E23" s="75" t="inlineStr">
         <is>
           <t>Step source CR0 / CR1 / LR / dst itself  [corner]</t>
         </is>
       </c>
-      <c r="F23" s="75" t="inlineStr">
+      <c r="F23" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G23" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H23" s="75" t="inlineStr">
+      <c r="G23" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H23" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2712,22 +2742,22 @@
       <c r="B24" s="77" t="n"/>
       <c r="C24" s="77" t="n"/>
       <c r="D24" s="77" t="n"/>
-      <c r="E24" s="74" t="inlineStr">
+      <c r="E24" s="75" t="inlineStr">
         <is>
           <t>Pointer walk: repeated INC.MODP2 over many words (circular buffer)  [standard]</t>
         </is>
       </c>
-      <c r="F24" s="75" t="inlineStr">
+      <c r="F24" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G24" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H24" s="75" t="inlineStr">
+      <c r="G24" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H24" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2769,12 +2799,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G25" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H25" s="71" t="inlineStr">
+      <c r="G25" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H25" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2800,12 +2830,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G26" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H26" s="71" t="inlineStr">
+      <c r="G26" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H26" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2826,17 +2856,17 @@
           <t>Long repeated INC / DEC on the same LR (counter)  [standard]</t>
         </is>
       </c>
-      <c r="F27" s="71" t="inlineStr">
+      <c r="F27" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G27" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H27" s="71" t="inlineStr">
+      <c r="G27" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H27" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2848,42 +2878,42 @@
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="72" t="inlineStr">
+      <c r="A28" s="73" t="inlineStr">
         <is>
           <t>ADB-01</t>
         </is>
       </c>
-      <c r="B28" s="73" t="inlineStr">
+      <c r="B28" s="74" t="inlineStr">
         <is>
           <t>LR ops: ADDB / ADDBI</t>
         </is>
       </c>
-      <c r="C28" s="74" t="inlineStr">
+      <c r="C28" s="75" t="inlineStr">
         <is>
           <t>The module shall add the signed byte (src_b[7:0] for ADDB, imm for ADDBI) to each of the 8 bytes of LRDn, saturating each byte to [0,255].</t>
         </is>
       </c>
-      <c r="D28" s="74" t="inlineStr">
+      <c r="D28" s="75" t="inlineStr">
         <is>
           <t>LRDn = LR(n+1):LR(n). Byte order inside the pair — Spec Questions Q10.</t>
         </is>
       </c>
-      <c r="E28" s="74" t="inlineStr">
+      <c r="E28" s="75" t="inlineStr">
         <is>
           <t>Random pair content and random signed byte  [standard]</t>
         </is>
       </c>
-      <c r="F28" s="75" t="inlineStr">
+      <c r="F28" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G28" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H28" s="75" t="inlineStr">
+      <c r="G28" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H28" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2899,22 +2929,22 @@
       <c r="B29" s="76" t="n"/>
       <c r="C29" s="76" t="n"/>
       <c r="D29" s="76" t="n"/>
-      <c r="E29" s="74" t="inlineStr">
+      <c r="E29" s="75" t="inlineStr">
         <is>
           <t>Saturation class: bytes and value biased to 0 / 255 / ±127 / -128, mixed saturating and non-saturating bytes in one op  [corner]</t>
         </is>
       </c>
-      <c r="F29" s="75" t="inlineStr">
+      <c r="F29" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G29" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H29" s="75" t="inlineStr">
+      <c r="G29" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H29" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2930,22 +2960,22 @@
       <c r="B30" s="76" t="n"/>
       <c r="C30" s="76" t="n"/>
       <c r="D30" s="76" t="n"/>
-      <c r="E30" s="74" t="inlineStr">
+      <c r="E30" s="75" t="inlineStr">
         <is>
           <t>Operand decode class: ADDB src_b with non-zero upper bits; ADDBI imm in both 0..255 and signed spelling  [corner]</t>
         </is>
       </c>
-      <c r="F30" s="75" t="inlineStr">
+      <c r="F30" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G30" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H30" s="75" t="inlineStr">
+      <c r="G30" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H30" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -2961,22 +2991,22 @@
       <c r="B31" s="77" t="n"/>
       <c r="C31" s="77" t="n"/>
       <c r="D31" s="77" t="n"/>
-      <c r="E31" s="74" t="inlineStr">
+      <c r="E31" s="75" t="inlineStr">
         <is>
           <t>Pair addressing: every LRD0..LRD14, only LR(n) and LR(n+1) change; src_b inside the dest pair  [standard]</t>
         </is>
       </c>
-      <c r="F31" s="75" t="inlineStr">
+      <c r="F31" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G31" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H31" s="75" t="inlineStr">
+      <c r="G31" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H31" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3032,12 +3062,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G33" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H33" s="71" t="inlineStr">
+      <c r="G33" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H33" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3058,17 +3088,17 @@
           <t>Words with empty lanes (all 3 empty, or only some)  [corner]</t>
         </is>
       </c>
-      <c r="F34" s="71" t="inlineStr">
+      <c r="F34" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G34" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H34" s="71" t="inlineStr">
+      <c r="G34" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H34" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3089,17 +3119,17 @@
           <t>Words with several ADDB/ADDBI in one word (each one writes 2 registers, so up to 6 registers change — Q4)  [corner]</t>
         </is>
       </c>
-      <c r="F35" s="71" t="inlineStr">
+      <c r="F35" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G35" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H35" s="71" t="inlineStr">
+      <c r="G35" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H35" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3111,42 +3141,42 @@
       </c>
     </row>
     <row r="36" ht="85" customHeight="1">
-      <c r="A36" s="72" t="inlineStr">
+      <c r="A36" s="73" t="inlineStr">
         <is>
           <t>LAN-02</t>
         </is>
       </c>
-      <c r="B36" s="73" t="inlineStr">
+      <c r="B36" s="74" t="inlineStr">
         <is>
           <t>LR lanes (x3)</t>
         </is>
       </c>
-      <c r="C36" s="74" t="inlineStr">
+      <c r="C36" s="75" t="inlineStr">
         <is>
           <t>All lanes shall read their input registers as they were at the START of the cycle, never the result of another lane in the same word.</t>
         </is>
       </c>
-      <c r="D36" s="74" t="inlineStr">
+      <c r="D36" s="75" t="inlineStr">
         <is>
           <t>Example word: lane0 = INC LR1 5, lane1 = ADD LR2 LR1 CR0. Lane1 must use the OLD LR1 (before +5), because lane0's write only becomes visible in the next word. Another example: lane0 = ADD LR0 LR1 CR0 and lane1 = ADD LR1 LR0 CR0 in one word swaps the two registers.</t>
         </is>
       </c>
-      <c r="E36" s="74" t="inlineStr">
+      <c r="E36" s="75" t="inlineStr">
         <is>
           <t>Random words where one lane reads a register that another lane writes in the same word (any lane pair, any command)  [corner]</t>
         </is>
       </c>
-      <c r="F36" s="75" t="inlineStr">
+      <c r="F36" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G36" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H36" s="75" t="inlineStr">
+      <c r="G36" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H36" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3188,12 +3218,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G37" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H37" s="71" t="inlineStr">
+      <c r="G37" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H37" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3205,42 +3235,42 @@
       </c>
     </row>
     <row r="38" ht="59" customHeight="1">
-      <c r="A38" s="72" t="inlineStr">
+      <c r="A38" s="73" t="inlineStr">
         <is>
           <t>TIM-01</t>
         </is>
       </c>
-      <c r="B38" s="73" t="inlineStr">
+      <c r="B38" s="74" t="inlineStr">
         <is>
           <t>LR hazards &amp; timing</t>
         </is>
       </c>
-      <c r="C38" s="74" t="inlineStr">
+      <c r="C38" s="75" t="inlineStr">
         <is>
           <t>A value written to an LR in word N shall be usable by the LR lanes in word N+1 (and any later word), with no gap.</t>
         </is>
       </c>
-      <c r="D38" s="74" t="inlineStr">
+      <c r="D38" s="75" t="inlineStr">
         <is>
           <t>Example: word N: SET LR3 #5. Word N+1: ADD LR4 LR3 CR1 must see LR3 = 5. This is the most common pattern in real code (counters, pointers), so it must work back-to-back.</t>
         </is>
       </c>
-      <c r="E38" s="74" t="inlineStr">
+      <c r="E38" s="75" t="inlineStr">
         <is>
           <t>Random chains of words where each word uses a register written 1, 2, 3 … words earlier; random command in producer and consumer  [standard]</t>
         </is>
       </c>
-      <c r="F38" s="75" t="inlineStr">
+      <c r="F38" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G38" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H38" s="75" t="inlineStr">
+      <c r="G38" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H38" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3282,12 +3312,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G39" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H39" s="71" t="inlineStr">
+      <c r="G39" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H39" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3299,42 +3329,42 @@
       </c>
     </row>
     <row r="40" ht="98" customHeight="1">
-      <c r="A40" s="72" t="inlineStr">
+      <c r="A40" s="73" t="inlineStr">
         <is>
           <t>TIM-03</t>
         </is>
       </c>
-      <c r="B40" s="73" t="inlineStr">
+      <c r="B40" s="74" t="inlineStr">
         <is>
           <t>LR hazards &amp; timing</t>
         </is>
       </c>
-      <c r="C40" s="74" t="inlineStr">
+      <c r="C40" s="75" t="inlineStr">
         <is>
           <t>At a branch the chip fetches both the next word and the branch target. Only the chosen word may have any effect; the other one shall have none.</t>
         </is>
       </c>
-      <c r="D40" s="74" t="inlineStr">
+      <c r="D40" s="75" t="inlineStr">
         <is>
           <t>Example: BEQ … target. The word at PC+1 holds INC LR5, the word at the target holds INC LR6. If the branch is taken, LR5 must NOT change; if not taken, LR6 must NOT change. The same for loads and the other stage slots. The branch word's own LR / load / stage slots always run, taken or not.</t>
         </is>
       </c>
-      <c r="E40" s="74" t="inlineStr">
+      <c r="E40" s="75" t="inlineStr">
         <is>
           <t>Random branches (taken and not taken) where both candidate words carry LR writes, loads and stage slots  [corner]</t>
         </is>
       </c>
-      <c r="F40" s="75" t="inlineStr">
+      <c r="F40" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G40" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H40" s="75" t="inlineStr">
+      <c r="G40" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H40" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3371,17 +3401,17 @@
           <t>Random programs mixing single-register and pair (LRD) access across all LRs and CRs  [standard]</t>
         </is>
       </c>
-      <c r="F41" s="71" t="inlineStr">
+      <c r="F41" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G41" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H41" s="71" t="inlineStr">
+      <c r="G41" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H41" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3393,42 +3423,42 @@
       </c>
     </row>
     <row r="42" ht="46" customHeight="1">
-      <c r="A42" s="72" t="inlineStr">
+      <c r="A42" s="73" t="inlineStr">
         <is>
           <t>LRF-02</t>
         </is>
       </c>
-      <c r="B42" s="73" t="inlineStr">
+      <c r="B42" s="74" t="inlineStr">
         <is>
           <t>LR / CR state &amp; reset</t>
         </is>
       </c>
-      <c r="C42" s="74" t="inlineStr">
+      <c r="C42" s="75" t="inlineStr">
         <is>
           <t>On reset the module shall go back to PC 0 and throw away any LR writes that were still in progress.</t>
         </is>
       </c>
-      <c r="D42" s="74" t="inlineStr">
+      <c r="D42" s="75" t="inlineStr">
         <is>
           <t>Reset value of the LRs is not written in the spec (Q6), so only the PC / no-late-write part can be checked now.</t>
         </is>
       </c>
-      <c r="E42" s="74" t="inlineStr">
+      <c r="E42" s="75" t="inlineStr">
         <is>
           <t>Reset applied at a random moment: in the middle of a program, in the cycle of a branch, after HALT; short and long pulses  [corner]</t>
         </is>
       </c>
-      <c r="F42" s="75" t="inlineStr">
+      <c r="F42" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G42" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H42" s="75" t="inlineStr">
+      <c r="G42" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H42" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3484,12 +3514,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G44" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H44" s="71" t="inlineStr">
+      <c r="G44" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H44" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3515,12 +3545,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G45" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H45" s="71" t="inlineStr">
+      <c r="G45" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H45" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3541,17 +3571,17 @@
           <t>Same register as both operands; LR k vs CR k  [corner]</t>
         </is>
       </c>
-      <c r="F46" s="71" t="inlineStr">
+      <c r="F46" s="79" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G46" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H46" s="71" t="inlineStr">
+      <c r="G46" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H46" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3563,42 +3593,42 @@
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="72" t="inlineStr">
+      <c r="A47" s="73" t="inlineStr">
         <is>
           <t>CND-02</t>
         </is>
       </c>
-      <c r="B47" s="73" t="inlineStr">
+      <c r="B47" s="74" t="inlineStr">
         <is>
           <t>COND: branches</t>
         </is>
       </c>
-      <c r="C47" s="74" t="inlineStr">
+      <c r="C47" s="75" t="inlineStr">
         <is>
           <t>The module shall always branch to reg[6:0] when BR is issued.</t>
         </is>
       </c>
-      <c r="D47" s="74" t="inlineStr">
+      <c r="D47" s="75" t="inlineStr">
         <is>
           <t>Upper bits of reg ignored (PC_W = 7).</t>
         </is>
       </c>
-      <c r="E47" s="74" t="inlineStr">
+      <c r="E47" s="75" t="inlineStr">
         <is>
           <t>Random reg (LR / CR) targets  [standard]</t>
         </is>
       </c>
-      <c r="F47" s="75" t="inlineStr">
+      <c r="F47" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G47" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H47" s="75" t="inlineStr">
+      <c r="G47" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H47" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3614,22 +3644,22 @@
       <c r="B48" s="77" t="n"/>
       <c r="C48" s="77" t="n"/>
       <c r="D48" s="77" t="n"/>
-      <c r="E48" s="74" t="inlineStr">
+      <c r="E48" s="75" t="inlineStr">
         <is>
           <t>Targets at the bank edges and reg values with upper bits set  [corner]</t>
         </is>
       </c>
-      <c r="F48" s="75" t="inlineStr">
+      <c r="F48" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G48" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H48" s="75" t="inlineStr">
+      <c r="G48" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H48" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3671,12 +3701,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G49" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H49" s="71" t="inlineStr">
+      <c r="G49" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H49" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3702,12 +3732,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G50" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H50" s="71" t="inlineStr">
+      <c r="G50" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H50" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3728,17 +3758,17 @@
           <t>HALT at the first and at the last bank entry  [corner]</t>
         </is>
       </c>
-      <c r="F51" s="71" t="inlineStr">
+      <c r="F51" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G51" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H51" s="71" t="inlineStr">
+      <c r="G51" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H51" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3750,38 +3780,38 @@
       </c>
     </row>
     <row r="52" ht="46" customHeight="1">
-      <c r="A52" s="72" t="inlineStr">
+      <c r="A52" s="73" t="inlineStr">
         <is>
           <t>HLT-02</t>
         </is>
       </c>
-      <c r="B52" s="73" t="inlineStr">
+      <c r="B52" s="74" t="inlineStr">
         <is>
           <t>COND: HALT</t>
         </is>
       </c>
-      <c r="C52" s="74" t="inlineStr">
+      <c r="C52" s="75" t="inlineStr">
         <is>
           <t>The module shall execute and dispatch every other slot of the HALT word exactly once.</t>
         </is>
       </c>
-      <c r="D52" s="74" t="n"/>
-      <c r="E52" s="74" t="inlineStr">
+      <c r="D52" s="75" t="n"/>
+      <c r="E52" s="75" t="inlineStr">
         <is>
           <t>HALT word with random LR lanes, load and MULT / ACC / AAQ / STORE slots  [standard]</t>
         </is>
       </c>
-      <c r="F52" s="75" t="inlineStr">
+      <c r="F52" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G52" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H52" s="75" t="inlineStr">
+      <c r="G52" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H52" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3818,17 +3848,17 @@
           <t>Back-to-back kernels with different programs  [standard]</t>
         </is>
       </c>
-      <c r="F53" s="71" t="inlineStr">
+      <c r="F53" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G53" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H53" s="71" t="inlineStr">
+      <c r="G53" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H53" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3884,12 +3914,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G55" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H55" s="71" t="inlineStr">
+      <c r="G55" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H55" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3915,12 +3945,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G56" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H56" s="71" t="inlineStr">
+      <c r="G56" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H56" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3932,38 +3962,38 @@
       </c>
     </row>
     <row r="57" ht="33" customHeight="1">
-      <c r="A57" s="72" t="inlineStr">
+      <c r="A57" s="73" t="inlineStr">
         <is>
           <t>FET-02</t>
         </is>
       </c>
-      <c r="B57" s="73" t="inlineStr">
+      <c r="B57" s="74" t="inlineStr">
         <is>
           <t>Fetch / PC</t>
         </is>
       </c>
-      <c r="C57" s="74" t="inlineStr">
+      <c r="C57" s="75" t="inlineStr">
         <is>
           <t>The module shall execute loops and nested loops driven by LR counters.</t>
         </is>
       </c>
-      <c r="D57" s="74" t="n"/>
-      <c r="E57" s="74" t="inlineStr">
+      <c r="D57" s="75" t="n"/>
+      <c r="E57" s="75" t="inlineStr">
         <is>
           <t>Random trip counts incl. 0 and 1, nesting 1..3 levels  [standard]</t>
         </is>
       </c>
-      <c r="F57" s="75" t="inlineStr">
+      <c r="F57" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G57" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H57" s="75" t="inlineStr">
+      <c r="G57" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H57" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4005,12 +4035,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G58" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H58" s="71" t="inlineStr">
+      <c r="G58" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H58" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4061,17 +4091,17 @@
           <t>Random words, random NOP slots  [standard]</t>
         </is>
       </c>
-      <c r="F60" s="71" t="inlineStr">
+      <c r="F60" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G60" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H60" s="71" t="inlineStr">
+      <c r="G60" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H60" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4083,42 +4113,42 @@
       </c>
     </row>
     <row r="61" ht="59" customHeight="1">
-      <c r="A61" s="72" t="inlineStr">
+      <c r="A61" s="73" t="inlineStr">
         <is>
           <t>DSP-02</t>
         </is>
       </c>
-      <c r="B61" s="73" t="inlineStr">
+      <c r="B61" s="74" t="inlineStr">
         <is>
           <t>Dispatch &amp; XMEM load</t>
         </is>
       </c>
-      <c r="C61" s="74" t="inlineStr">
+      <c r="C61" s="75" t="inlineStr">
         <is>
           <t>The module shall pack on the buses the post-LR-write value of every CR/LR operand, while its own LR/branch reads use the snapshot.</t>
         </is>
       </c>
-      <c r="D61" s="74" t="inlineStr">
+      <c r="D61" s="75" t="inlineStr">
         <is>
           <t>Spec §5 / §7.</t>
         </is>
       </c>
-      <c r="E61" s="74" t="inlineStr">
+      <c r="E61" s="75" t="inlineStr">
         <is>
           <t>Words where a bus operand LR is written by a lane in the same word (any opcode, lane, bus)  [corner]</t>
         </is>
       </c>
-      <c r="F61" s="75" t="inlineStr">
+      <c r="F61" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G61" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H61" s="75" t="inlineStr">
+      <c r="G61" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H61" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4156,12 +4186,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G62" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H62" s="71" t="inlineStr">
+      <c r="G62" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H62" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4187,12 +4217,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G63" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H63" s="71" t="inlineStr">
+      <c r="G63" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H63" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4213,17 +4243,17 @@
           <t>Sum overflow past XMEM_ADDR_W and negative offsets  [corner]</t>
         </is>
       </c>
-      <c r="F64" s="71" t="inlineStr">
+      <c r="F64" s="78" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G64" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H64" s="71" t="inlineStr">
+      <c r="G64" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H64" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4235,38 +4265,38 @@
       </c>
     </row>
     <row r="65" ht="33" customHeight="1">
-      <c r="A65" s="72" t="inlineStr">
+      <c r="A65" s="73" t="inlineStr">
         <is>
           <t>DSP-04</t>
         </is>
       </c>
-      <c r="B65" s="73" t="inlineStr">
+      <c r="B65" s="74" t="inlineStr">
         <is>
           <t>Dispatch &amp; XMEM load</t>
         </is>
       </c>
-      <c r="C65" s="74" t="inlineStr">
+      <c r="C65" s="75" t="inlineStr">
         <is>
           <t>The module shall assert xmem_read_en only for non-NOP loads of the executed path.</t>
         </is>
       </c>
-      <c r="D65" s="74" t="n"/>
-      <c r="E65" s="74" t="inlineStr">
+      <c r="D65" s="75" t="n"/>
+      <c r="E65" s="75" t="inlineStr">
         <is>
           <t>Random load density (every word, sparse, none), incl. loads in branch and HALT words  [standard]</t>
         </is>
       </c>
-      <c r="F65" s="75" t="inlineStr">
+      <c r="F65" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G65" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H65" s="75" t="inlineStr">
+      <c r="G65" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H65" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4282,22 +4312,22 @@
       <c r="B66" s="77" t="n"/>
       <c r="C66" s="77" t="n"/>
       <c r="D66" s="77" t="n"/>
-      <c r="E66" s="74" t="inlineStr">
+      <c r="E66" s="75" t="inlineStr">
         <is>
           <t>Load only in the non-selected candidate → no read  [corner]</t>
         </is>
       </c>
-      <c r="F66" s="75" t="inlineStr">
+      <c r="F66" s="71" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G66" s="75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H66" s="75" t="inlineStr">
+      <c r="G66" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H66" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4353,12 +4383,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G68" s="71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H68" s="71" t="inlineStr">
+      <c r="G68" s="72" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H68" s="72" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4482,14 +4512,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="78" t="inlineStr">
+      <c r="A1" s="80" t="inlineStr">
         <is>
           <t>Spec Questions — to close with the designer before the VP is built</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="79" t="inlineStr">
+      <c r="A2" s="81" t="inlineStr">
         <is>
           <t>Findings from reading specs/stage-control: inconsistencies and gaps that block exact checker expectations.</t>
         </is>
@@ -4523,405 +4553,405 @@
       </c>
     </row>
     <row r="5" ht="47" customHeight="1">
-      <c r="A5" s="80" t="inlineStr">
+      <c r="A5" s="82" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="B5" s="81" t="inlineStr">
+      <c r="B5" s="83" t="inlineStr">
         <is>
           <t>§10 intro, §8, Summary table</t>
         </is>
       </c>
-      <c r="C5" s="81" t="inlineStr">
+      <c r="C5" s="83" t="inlineStr">
         <is>
           <t>Intro says '11 mnemonics: four LR ops + seven branches'; §8 lists LR ops 'SET/ADD/SUB/INC.MODP2'. The table and §4 list 8 LR ops and 5 branches + HALT (6 COND).</t>
         </is>
       </c>
-      <c r="D5" s="81" t="inlineStr">
+      <c r="D5" s="83" t="inlineStr">
         <is>
           <t>Stale text – risk that the AL misses or invents an opcode.</t>
         </is>
       </c>
-      <c r="E5" s="81" t="inlineStr">
+      <c r="E5" s="83" t="inlineStr">
         <is>
           <t>Confirm the final opcode set is 8 LR + 5 branch + HALT.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="80" t="inlineStr">
+      <c r="A6" s="82" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="B6" s="81" t="inlineStr">
+      <c r="B6" s="83" t="inlineStr">
         <is>
           <t>§2 diagram vs §4</t>
         </is>
       </c>
-      <c r="C6" s="81" t="inlineStr">
+      <c r="C6" s="83" t="inlineStr">
         <is>
           <t>Diagram says 'CR file 2 x 16 x 20bit' and 'LR file 16 x 20bit'; §4 REG_WIDTH = 32.</t>
         </is>
       </c>
-      <c r="D6" s="81" t="inlineStr">
+      <c r="D6" s="83" t="inlineStr">
         <is>
           <t>Width decides all overflow / wrap corners (0xFFFFFFFF vs 20-bit).</t>
         </is>
       </c>
-      <c r="E6" s="81" t="inlineStr">
+      <c r="E6" s="83" t="inlineStr">
         <is>
           <t>Is every CR/LR 32 bit? (AL assumes 32.)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="80" t="inlineStr">
+      <c r="A7" s="82" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="B7" s="81" t="inlineStr">
+      <c r="B7" s="83" t="inlineStr">
         <is>
           <t>§6.3 vs §10.2</t>
         </is>
       </c>
-      <c r="C7" s="81" t="inlineStr">
+      <c r="C7" s="83" t="inlineStr">
         <is>
           <t>§6.3 / pseudo-code use next_pc = label (absolute). §10.2 says 'label is a relative offset resolved by the assembler'.</t>
         </is>
       </c>
-      <c r="D7" s="81" t="inlineStr">
+      <c r="D7" s="83" t="inlineStr">
         <is>
           <t>Absolute vs relative changes target computation, wrap and range corners (FET-01).</t>
         </is>
       </c>
-      <c r="E7" s="81" t="inlineStr">
+      <c r="E7" s="83" t="inlineStr">
         <is>
           <t>Does the label field in IMEM hold an absolute address or a PC-relative offset?</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="80" t="inlineStr">
+      <c r="A8" s="82" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="B8" s="81" t="inlineStr">
+      <c r="B8" s="83" t="inlineStr">
         <is>
           <t>§1, §10.1.7</t>
         </is>
       </c>
-      <c r="C8" s="81" t="inlineStr">
+      <c r="C8" s="83" t="inlineStr">
         <is>
           <t>'Up to three local-register writes per cycle', but ADDB/ADDBI write two LRs (the pair) each → up to six.</t>
         </is>
       </c>
-      <c r="D8" s="81" t="inlineStr">
+      <c r="D8" s="83" t="inlineStr">
         <is>
           <t>Number of LR write ports / pair conflicts (LAN-01, SYS-02).</t>
         </is>
       </c>
-      <c r="E8" s="81" t="inlineStr">
+      <c r="E8" s="83" t="inlineStr">
         <is>
           <t>Is the LR file 6-write? What happens if pairs overlap other lanes?</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="80" t="inlineStr">
+      <c r="A9" s="82" t="inlineStr">
         <is>
           <t>Q5</t>
         </is>
       </c>
-      <c r="B9" s="81" t="inlineStr">
+      <c r="B9" s="83" t="inlineStr">
         <is>
           <t>§10.1 (self-reference '§10')</t>
         </is>
       </c>
-      <c r="C9" s="81" t="inlineStr">
+      <c r="C9" s="83" t="inlineStr">
         <is>
           <t>'Programs must not target the same destination LR from two lanes' – no hardware behavior stated.</t>
         </is>
       </c>
-      <c r="D9" s="81" t="inlineStr">
+      <c r="D9" s="83" t="inlineStr">
         <is>
           <t>Needed to turn SYS-02 into a checker (lane priority? last lane wins? undefined?).</t>
         </is>
       </c>
-      <c r="E9" s="81" t="inlineStr">
+      <c r="E9" s="83" t="inlineStr">
         <is>
           <t>Define the behavior or declare it undefined/ignored.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="80" t="inlineStr">
+      <c r="A10" s="82" t="inlineStr">
         <is>
           <t>Q6</t>
         </is>
       </c>
-      <c r="B10" s="81" t="inlineStr">
+      <c r="B10" s="83" t="inlineStr">
         <is>
           <t>§3.1</t>
         </is>
       </c>
-      <c r="C10" s="81" t="inlineStr">
+      <c r="C10" s="83" t="inlineStr">
         <is>
           <t>Reset 'clears any pending LR writes' – LR values after reset are not stated.</t>
         </is>
       </c>
-      <c r="D10" s="81" t="inlineStr">
+      <c r="D10" s="83" t="inlineStr">
         <is>
           <t>LRF-02 cannot check the post-reset LR value.</t>
         </is>
       </c>
-      <c r="E10" s="81" t="inlineStr">
+      <c r="E10" s="83" t="inlineStr">
         <is>
           <t>Are LR0..LR15 reset to 0? What is a 'pending LR write'?</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="80" t="inlineStr">
+      <c r="A11" s="82" t="inlineStr">
         <is>
           <t>Q7</t>
         </is>
       </c>
-      <c r="B11" s="81" t="inlineStr">
+      <c r="B11" s="83" t="inlineStr">
         <is>
           <t>§5, §10.1</t>
         </is>
       </c>
-      <c r="C11" s="81" t="inlineStr">
+      <c r="C11" s="83" t="inlineStr">
         <is>
           <t>No LR-slot NOP is mentioned (only COND/load NOP).</t>
         </is>
       </c>
-      <c r="D11" s="81" t="inlineStr">
+      <c r="D11" s="83" t="inlineStr">
         <is>
           <t>LAN-01 assumes an LR NOP encoding.</t>
         </is>
       </c>
-      <c r="E11" s="81" t="inlineStr">
+      <c r="E11" s="83" t="inlineStr">
         <is>
           <t>How is an unused LR lane encoded?</t>
         </is>
       </c>
     </row>
     <row r="12" ht="47" customHeight="1">
-      <c r="A12" s="80" t="inlineStr">
+      <c r="A12" s="82" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="B12" s="81" t="inlineStr">
+      <c r="B12" s="83" t="inlineStr">
         <is>
           <t>§7.1, §9</t>
         </is>
       </c>
-      <c r="C12" s="81" t="inlineStr">
+      <c r="C12" s="83" t="inlineStr">
         <is>
           <t>xmem_read_en is gated by '!bubble' and refers to '§9.2'; §9 says no hazard interlocks exist and §9.2 does not exist.</t>
         </is>
       </c>
-      <c r="D12" s="81" t="inlineStr">
+      <c r="D12" s="83" t="inlineStr">
         <is>
           <t>Memory-wait / stall behavior is undefined (group MEM is a placeholder).</t>
         </is>
       </c>
-      <c r="E12" s="81" t="inlineStr">
+      <c r="E12" s="83" t="inlineStr">
         <is>
           <t>Provide the updated wait/stall mechanism (stall input? bubble counter? who holds PC / LR commit?).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="80" t="inlineStr">
+      <c r="A13" s="82" t="inlineStr">
         <is>
           <t>Q9</t>
         </is>
       </c>
-      <c r="B13" s="81" t="inlineStr">
+      <c r="B13" s="83" t="inlineStr">
         <is>
           <t>§10.1.4</t>
         </is>
       </c>
-      <c r="C13" s="81" t="inlineStr">
+      <c r="C13" s="83" t="inlineStr">
         <is>
           <t>INC.MODP2 k is 4 bits encoded k-1, semantic range 1..9; encodings 9..15 are not described.</t>
         </is>
       </c>
-      <c r="D13" s="81" t="inlineStr">
+      <c r="D13" s="83" t="inlineStr">
         <is>
           <t>Expected result for illegal k (SYS-02).</t>
         </is>
       </c>
-      <c r="E13" s="81" t="inlineStr">
+      <c r="E13" s="83" t="inlineStr">
         <is>
           <t>Is the encoding legal-checked, saturated or just masked?</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="80" t="inlineStr">
+      <c r="A14" s="82" t="inlineStr">
         <is>
           <t>Q10</t>
         </is>
       </c>
-      <c r="B14" s="81" t="inlineStr">
+      <c r="B14" s="83" t="inlineStr">
         <is>
           <t>§10.1.7-8</t>
         </is>
       </c>
-      <c r="C14" s="81" t="inlineStr">
+      <c r="C14" s="83" t="inlineStr">
         <is>
           <t>Byte-element order inside LRDn is not stated (which LR holds elements 0-3; element 0 = bits [7:0]?).</t>
         </is>
       </c>
-      <c r="D14" s="81" t="inlineStr">
+      <c r="D14" s="83" t="inlineStr">
         <is>
           <t>ADB-01 checker needs the exact lane mapping.</t>
         </is>
       </c>
-      <c r="E14" s="81" t="inlineStr">
+      <c r="E14" s="83" t="inlineStr">
         <is>
           <t>Confirm element i = LRD bits [8i+7:8i], LR(n) = low half.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="47" customHeight="1">
-      <c r="A15" s="80" t="inlineStr">
+      <c r="A15" s="82" t="inlineStr">
         <is>
           <t>Q11</t>
         </is>
       </c>
-      <c r="B15" s="81" t="inlineStr">
+      <c r="B15" s="83" t="inlineStr">
         <is>
           <t>§1, §7.1</t>
         </is>
       </c>
-      <c r="C15" s="81" t="inlineStr">
+      <c r="C15" s="83" t="inlineStr">
         <is>
           <t>The load slot 'has no opcode' yet 'writes into R0/R1/R_CYCLIC/R_MASK' – the destination register is not visible on the CTRL ports (only addr + en).</t>
         </is>
       </c>
-      <c r="D15" s="81" t="inlineStr">
+      <c r="D15" s="83" t="inlineStr">
         <is>
           <t>Whether CTRL must forward a destination-select with the load.</t>
         </is>
       </c>
-      <c r="E15" s="81" t="inlineStr">
+      <c r="E15" s="83" t="inlineStr">
         <is>
           <t>Is the destination select part of xmem_read_* or of mult_vliw_bus?</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="80" t="inlineStr">
+      <c r="A16" s="82" t="inlineStr">
         <is>
           <t>Q12</t>
         </is>
       </c>
-      <c r="B16" s="81" t="inlineStr">
+      <c r="B16" s="83" t="inlineStr">
         <is>
           <t>§6.3, §4</t>
         </is>
       </c>
-      <c r="C16" s="81" t="inlineStr">
+      <c r="C16" s="83" t="inlineStr">
         <is>
           <t>PC_W = 7 (bank depth 128) but IMEM_DEPTH = 256. Behavior of PC+1 past the last entry is unspecified.</t>
         </is>
       </c>
-      <c r="D16" s="81" t="inlineStr">
+      <c r="D16" s="83" t="inlineStr">
         <is>
           <t>Illegal PC range (SYS-02).</t>
         </is>
       </c>
-      <c r="E16" s="81" t="inlineStr">
+      <c r="E16" s="83" t="inlineStr">
         <is>
           <t>Does PC wrap, stop, or is it illegal?</t>
         </is>
       </c>
     </row>
     <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="80" t="inlineStr">
+      <c r="A17" s="82" t="inlineStr">
         <is>
           <t>Q13</t>
         </is>
       </c>
-      <c r="B17" s="81" t="inlineStr">
+      <c r="B17" s="83" t="inlineStr">
         <is>
           <t>§6.4, §3 black box</t>
         </is>
       </c>
-      <c r="C17" s="81" t="inlineStr">
+      <c r="C17" s="83" t="inlineStr">
         <is>
           <t>Spec cites kernel_done, IPU-EXEC-13 (restart at PC 0) and imem_bank_sel, but none of them is a port of CTRL.</t>
         </is>
       </c>
-      <c r="D17" s="81" t="inlineStr">
+      <c r="D17" s="83" t="inlineStr">
         <is>
           <t>HLT-03: how are kernel start / done observed and driven?</t>
         </is>
       </c>
-      <c r="E17" s="81" t="inlineStr">
+      <c r="E17" s="83" t="inlineStr">
         <is>
           <t>Provide the start / done interface (APB register? side-band?).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="80" t="inlineStr">
+      <c r="A18" s="82" t="inlineStr">
         <is>
           <t>Q14</t>
         </is>
       </c>
-      <c r="B18" s="81" t="inlineStr">
+      <c r="B18" s="83" t="inlineStr">
         <is>
           <t>§8</t>
         </is>
       </c>
-      <c r="C18" s="81" t="inlineStr">
+      <c r="C18" s="83" t="inlineStr">
         <is>
           <t>'New active bank takes effect on the next CTRL fetch cycle' – behavior of a swap while a kernel is running is not defined.</t>
         </is>
       </c>
-      <c r="D18" s="81" t="inlineStr">
+      <c r="D18" s="83" t="inlineStr">
         <is>
           <t>Out of this AL revision (APB), but affects fetch coherence.</t>
         </is>
       </c>
-      <c r="E18" s="81" t="inlineStr">
+      <c r="E18" s="83" t="inlineStr">
         <is>
           <t>Is swap while running illegal?</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="80" t="inlineStr">
+      <c r="A19" s="82" t="inlineStr">
         <is>
           <t>Q15</t>
         </is>
       </c>
-      <c r="B19" s="81" t="inlineStr">
+      <c r="B19" s="83" t="inlineStr">
         <is>
           <t>§10.2</t>
         </is>
       </c>
-      <c r="C19" s="81" t="inlineStr">
+      <c r="C19" s="83" t="inlineStr">
         <is>
           <t>COND pseudo-code reads reg1 and reg2 for every op including BR / HALT; BR reg is also read from the snapshot.</t>
         </is>
       </c>
-      <c r="D19" s="81" t="inlineStr">
+      <c r="D19" s="83" t="inlineStr">
         <is>
           <t>TIM-02 for BR.</t>
         </is>
       </c>
-      <c r="E19" s="81" t="inlineStr">
+      <c r="E19" s="83" t="inlineStr">
         <is>
           <t>Confirm BR target reads the same prior-cycle snapshot as the compares.</t>
         </is>

</xml_diff>